<commit_message>
Fig 2 panel styling: axisless variants, TC50 cleanup, plasma colors, standalone legends
- Restyle TC50 dose-response (remove grid/title, black sigmoid, log10 x-axis, error bars, well exclusions)
- Add native axisless generation to O2, contractility, and waveform plot scripts
- Match waveform colors to contractility plasma colormap
- Export concentration legends as standalone PNGs (separate from plots)
- Set all 2D plots to 10x8 figsize (0.8 aspect ratio)
- Add generate_axisless_figures.py with monkey-patch + backfill for all figures
- Add axis scaling reference sheets and figure image catalog
- Regenerate all figure outputs with updated styling

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Output/PowerPoint_Figures/Fig_2/Fig_2d_data.xlsx
+++ b/Output/PowerPoint_Figures/Fig_2/Fig_2d_data.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,39 +418,39 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>SNR Bucket</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>% In Range (0-80%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>% Out of Range</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -479,7 +467,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -489,7 +477,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -506,7 +494,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -516,7 +504,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -533,7 +521,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -543,7 +531,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">
@@ -560,7 +548,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -570,7 +558,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="n">
@@ -587,7 +575,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -597,7 +585,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="n">
@@ -614,7 +602,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -624,7 +612,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="n">
@@ -641,7 +629,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -651,7 +639,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="n">
@@ -668,7 +656,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -678,7 +666,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="n">
@@ -695,7 +683,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -705,7 +693,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="n">
@@ -722,7 +710,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -732,7 +720,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="n">
@@ -749,7 +737,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -759,7 +747,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="n">
@@ -776,7 +764,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -786,7 +774,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
@@ -803,7 +791,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -813,7 +801,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="n">
@@ -830,7 +818,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -840,7 +828,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="n">
@@ -857,7 +845,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -867,7 +855,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="n">
@@ -884,7 +872,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -894,7 +882,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="n">
@@ -911,7 +899,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -921,7 +909,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="n">
@@ -938,7 +926,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -948,7 +936,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
       <c r="B20" t="n">
@@ -965,7 +953,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -975,7 +963,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
       <c r="B21" t="n">
@@ -992,7 +980,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1002,7 +990,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
       <c r="B22" t="n">
@@ -1019,7 +1007,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1029,7 +1017,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
       <c r="B23" t="n">
@@ -1046,7 +1034,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1056,7 +1044,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
       <c r="B24" t="n">
@@ -1073,7 +1061,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1083,7 +1071,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
       <c r="B25" t="n">
@@ -1100,7 +1088,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1110,7 +1098,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
       <c r="B26" t="n">
@@ -1127,7 +1115,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1137,7 +1125,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
       <c r="B27" t="n">
@@ -1154,7 +1142,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1164,7 +1152,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
       <c r="B28" t="n">
@@ -1181,7 +1169,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1191,7 +1179,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>27</v>
       </c>
       <c r="B29" t="n">
@@ -1208,7 +1196,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1218,7 +1206,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>28</v>
       </c>
       <c r="B30" t="n">
@@ -1235,7 +1223,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1245,7 +1233,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>29</v>
       </c>
       <c r="B31" t="n">
@@ -1262,7 +1250,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1272,7 +1260,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>30</v>
       </c>
       <c r="B32" t="n">
@@ -1289,7 +1277,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1299,7 +1287,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>31</v>
       </c>
       <c r="B33" t="n">
@@ -1316,7 +1304,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1326,7 +1314,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>32</v>
       </c>
       <c r="B34" t="n">
@@ -1343,7 +1331,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1353,7 +1341,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>33</v>
       </c>
       <c r="B35" t="n">
@@ -1370,7 +1358,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1380,7 +1368,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>34</v>
       </c>
       <c r="B36" t="n">
@@ -1397,7 +1385,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1407,7 +1395,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>35</v>
       </c>
       <c r="B37" t="n">
@@ -1424,7 +1412,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1434,7 +1422,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>36</v>
       </c>
       <c r="B38" t="n">
@@ -1451,7 +1439,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1461,7 +1449,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>37</v>
       </c>
       <c r="B39" t="n">
@@ -1478,7 +1466,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1488,7 +1476,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>38</v>
       </c>
       <c r="B40" t="n">
@@ -1505,7 +1493,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1515,7 +1503,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>39</v>
       </c>
       <c r="B41" t="n">
@@ -1532,7 +1520,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1542,7 +1530,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>40</v>
       </c>
       <c r="B42" t="n">
@@ -1559,7 +1547,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1569,7 +1557,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>41</v>
       </c>
       <c r="B43" t="n">
@@ -1586,7 +1574,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1596,7 +1584,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>42</v>
       </c>
       <c r="B44" t="n">
@@ -1613,7 +1601,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1623,7 +1611,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>43</v>
       </c>
       <c r="B45" t="n">
@@ -1640,7 +1628,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1650,7 +1638,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>44</v>
       </c>
       <c r="B46" t="n">
@@ -1667,7 +1655,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1677,7 +1665,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>45</v>
       </c>
       <c r="B47" t="n">
@@ -1694,7 +1682,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1704,7 +1692,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>46</v>
       </c>
       <c r="B48" t="n">
@@ -1721,7 +1709,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -1731,7 +1719,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>47</v>
       </c>
       <c r="B49" t="n">
@@ -1748,7 +1736,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1758,7 +1746,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>48</v>
       </c>
       <c r="B50" t="n">
@@ -1775,7 +1763,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -1785,7 +1773,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>49</v>
       </c>
       <c r="B51" t="n">
@@ -1802,7 +1790,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -1812,7 +1800,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>50</v>
       </c>
       <c r="B52" t="n">
@@ -1829,7 +1817,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -1839,7 +1827,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>51</v>
       </c>
       <c r="B53" t="n">
@@ -1856,7 +1844,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -1866,7 +1854,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>52</v>
       </c>
       <c r="B54" t="n">
@@ -1883,7 +1871,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -1893,7 +1881,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>53</v>
       </c>
       <c r="B55" t="n">
@@ -1910,7 +1898,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -1920,7 +1908,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>54</v>
       </c>
       <c r="B56" t="n">
@@ -1937,7 +1925,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -1947,7 +1935,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>55</v>
       </c>
       <c r="B57" t="n">
@@ -1964,7 +1952,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -1974,7 +1962,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>56</v>
       </c>
       <c r="B58" t="n">
@@ -1991,7 +1979,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2001,7 +1989,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>57</v>
       </c>
       <c r="B59" t="n">
@@ -2018,7 +2006,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2028,7 +2016,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>58</v>
       </c>
       <c r="B60" t="n">
@@ -2045,7 +2033,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2055,7 +2043,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>59</v>
       </c>
       <c r="B61" t="n">
@@ -2072,7 +2060,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2082,7 +2070,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>60</v>
       </c>
       <c r="B62" t="n">
@@ -2099,7 +2087,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2109,7 +2097,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>61</v>
       </c>
       <c r="B63" t="n">
@@ -2126,7 +2114,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2136,7 +2124,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>62</v>
       </c>
       <c r="B64" t="n">
@@ -2153,7 +2141,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2163,7 +2151,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>63</v>
       </c>
       <c r="B65" t="n">
@@ -2180,7 +2168,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2190,7 +2178,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>64</v>
       </c>
       <c r="B66" t="n">
@@ -2207,7 +2195,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2217,7 +2205,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>65</v>
       </c>
       <c r="B67" t="n">
@@ -2234,7 +2222,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2244,7 +2232,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>66</v>
       </c>
       <c r="B68" t="n">
@@ -2261,7 +2249,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2271,7 +2259,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>67</v>
       </c>
       <c r="B69" t="n">
@@ -2288,7 +2276,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2298,7 +2286,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>68</v>
       </c>
       <c r="B70" t="n">
@@ -2315,7 +2303,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2325,7 +2313,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>69</v>
       </c>
       <c r="B71" t="n">
@@ -2342,7 +2330,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2352,7 +2340,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>70</v>
       </c>
       <c r="B72" t="n">
@@ -2369,7 +2357,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2379,7 +2367,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>71</v>
       </c>
       <c r="B73" t="n">
@@ -2396,7 +2384,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2406,7 +2394,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>72</v>
       </c>
       <c r="B74" t="n">
@@ -2423,7 +2411,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2433,7 +2421,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>73</v>
       </c>
       <c r="B75" t="n">
@@ -2450,7 +2438,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2460,7 +2448,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>74</v>
       </c>
       <c r="B76" t="n">
@@ -2477,7 +2465,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2487,7 +2475,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>75</v>
       </c>
       <c r="B77" t="n">
@@ -2504,7 +2492,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -2514,7 +2502,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>76</v>
       </c>
       <c r="B78" t="n">
@@ -2531,7 +2519,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2541,7 +2529,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>77</v>
       </c>
       <c r="B79" t="n">
@@ -2558,7 +2546,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -2568,7 +2556,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>78</v>
       </c>
       <c r="B80" t="n">
@@ -2585,7 +2573,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -2595,7 +2583,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>79</v>
       </c>
       <c r="B81" t="n">
@@ -2612,7 +2600,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -2622,7 +2610,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>80</v>
       </c>
       <c r="B82" t="n">
@@ -2639,7 +2627,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2649,7 +2637,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>81</v>
       </c>
       <c r="B83" t="n">
@@ -2666,7 +2654,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -2676,7 +2664,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>82</v>
       </c>
       <c r="B84" t="n">
@@ -2693,7 +2681,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -2703,7 +2691,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>83</v>
       </c>
       <c r="B85" t="n">
@@ -2720,7 +2708,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -2730,7 +2718,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>84</v>
       </c>
       <c r="B86" t="n">
@@ -2747,7 +2735,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -2757,7 +2745,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>85</v>
       </c>
       <c r="B87" t="n">
@@ -2774,7 +2762,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -2784,7 +2772,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>86</v>
       </c>
       <c r="B88" t="n">
@@ -2801,7 +2789,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -2811,7 +2799,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>87</v>
       </c>
       <c r="B89" t="n">
@@ -2828,7 +2816,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -2838,7 +2826,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>88</v>
       </c>
       <c r="B90" t="n">
@@ -2855,7 +2843,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -2865,7 +2853,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>89</v>
       </c>
       <c r="B91" t="n">
@@ -2882,7 +2870,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -2892,7 +2880,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>90</v>
       </c>
       <c r="B92" t="n">
@@ -2909,7 +2897,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -2919,7 +2907,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>91</v>
       </c>
       <c r="B93" t="n">
@@ -2936,7 +2924,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -2946,7 +2934,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>92</v>
       </c>
       <c r="B94" t="n">
@@ -2963,7 +2951,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -2973,7 +2961,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" t="n">
         <v>93</v>
       </c>
       <c r="B95" t="n">
@@ -2990,7 +2978,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -3000,7 +2988,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" t="n">
         <v>94</v>
       </c>
       <c r="B96" t="n">
@@ -3017,7 +3005,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -3027,7 +3015,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" t="n">
         <v>95</v>
       </c>
       <c r="B97" t="n">
@@ -3044,7 +3032,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -3054,7 +3042,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" t="n">
         <v>96</v>
       </c>
       <c r="B98" t="n">
@@ -3071,7 +3059,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -3081,7 +3069,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" t="n">
         <v>97</v>
       </c>
       <c r="B99" t="n">
@@ -3098,7 +3086,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -3108,7 +3096,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" t="n">
         <v>98</v>
       </c>
       <c r="B100" t="n">
@@ -3125,7 +3113,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -3135,7 +3123,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" t="n">
         <v>99</v>
       </c>
       <c r="B101" t="n">
@@ -3152,7 +3140,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -3162,7 +3150,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" t="n">
         <v>100</v>
       </c>
       <c r="B102" t="n">
@@ -3179,7 +3167,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\Excel_Figures\snr_analysis.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/Excel_Figures/snr_analysis.xlsx</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -3203,39 +3191,39 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>SNR_Bucket_Lower (X)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Pct_In_Range_0_to_80 (Y)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Pct_Out_Range (Y)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Measurement_Count</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SNR_Bucket_Midpoint (X)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -3255,12 +3243,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -3280,12 +3268,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -3305,12 +3293,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">
@@ -3330,12 +3318,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="n">
@@ -3355,12 +3343,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="n">
@@ -3380,12 +3368,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="n">
@@ -3405,12 +3393,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="n">
@@ -3430,12 +3418,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="n">
@@ -3455,12 +3443,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="n">
@@ -3480,12 +3468,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="n">
@@ -3505,12 +3493,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="n">
@@ -3530,12 +3518,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
@@ -3555,12 +3543,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="n">
@@ -3580,12 +3568,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="n">
@@ -3605,12 +3593,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="n">
@@ -3630,12 +3618,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="n">
@@ -3655,12 +3643,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="n">
@@ -3680,12 +3668,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
       <c r="B20" t="n">
@@ -3705,12 +3693,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
       <c r="B21" t="n">
@@ -3730,12 +3718,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
       <c r="B22" t="n">
@@ -3755,12 +3743,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
       <c r="B23" t="n">
@@ -3780,12 +3768,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
       <c r="B24" t="n">
@@ -3805,12 +3793,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
       <c r="B25" t="n">
@@ -3830,12 +3818,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
       <c r="B26" t="n">
@@ -3855,12 +3843,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
       <c r="B27" t="n">
@@ -3880,12 +3868,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
       <c r="B28" t="n">
@@ -3905,12 +3893,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>27</v>
       </c>
       <c r="B29" t="n">
@@ -3930,12 +3918,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>28</v>
       </c>
       <c r="B30" t="n">
@@ -3955,12 +3943,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>29</v>
       </c>
       <c r="B31" t="n">
@@ -3980,12 +3968,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>30</v>
       </c>
       <c r="B32" t="n">
@@ -4005,12 +3993,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>31</v>
       </c>
       <c r="B33" t="n">
@@ -4030,12 +4018,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>32</v>
       </c>
       <c r="B34" t="n">
@@ -4055,12 +4043,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>33</v>
       </c>
       <c r="B35" t="n">
@@ -4080,12 +4068,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>34</v>
       </c>
       <c r="B36" t="n">
@@ -4105,12 +4093,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>35</v>
       </c>
       <c r="B37" t="n">
@@ -4130,12 +4118,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>36</v>
       </c>
       <c r="B38" t="n">
@@ -4155,12 +4143,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>37</v>
       </c>
       <c r="B39" t="n">
@@ -4180,12 +4168,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>38</v>
       </c>
       <c r="B40" t="n">
@@ -4205,12 +4193,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>39</v>
       </c>
       <c r="B41" t="n">
@@ -4230,12 +4218,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>40</v>
       </c>
       <c r="B42" t="n">
@@ -4255,12 +4243,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>41</v>
       </c>
       <c r="B43" t="n">
@@ -4280,12 +4268,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>42</v>
       </c>
       <c r="B44" t="n">
@@ -4305,12 +4293,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>43</v>
       </c>
       <c r="B45" t="n">
@@ -4330,12 +4318,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>44</v>
       </c>
       <c r="B46" t="n">
@@ -4355,12 +4343,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>45</v>
       </c>
       <c r="B47" t="n">
@@ -4380,12 +4368,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>46</v>
       </c>
       <c r="B48" t="n">
@@ -4405,12 +4393,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>47</v>
       </c>
       <c r="B49" t="n">
@@ -4430,12 +4418,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>48</v>
       </c>
       <c r="B50" t="n">
@@ -4455,12 +4443,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>49</v>
       </c>
       <c r="B51" t="n">
@@ -4480,12 +4468,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>50</v>
       </c>
       <c r="B52" t="n">
@@ -4505,12 +4493,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>51</v>
       </c>
       <c r="B53" t="n">
@@ -4530,12 +4518,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>52</v>
       </c>
       <c r="B54" t="n">
@@ -4555,12 +4543,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>53</v>
       </c>
       <c r="B55" t="n">
@@ -4580,12 +4568,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>54</v>
       </c>
       <c r="B56" t="n">
@@ -4605,12 +4593,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>55</v>
       </c>
       <c r="B57" t="n">
@@ -4630,12 +4618,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>56</v>
       </c>
       <c r="B58" t="n">
@@ -4655,12 +4643,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>57</v>
       </c>
       <c r="B59" t="n">
@@ -4680,12 +4668,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>58</v>
       </c>
       <c r="B60" t="n">
@@ -4705,12 +4693,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>59</v>
       </c>
       <c r="B61" t="n">
@@ -4730,12 +4718,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>60</v>
       </c>
       <c r="B62" t="n">
@@ -4755,12 +4743,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>61</v>
       </c>
       <c r="B63" t="n">
@@ -4780,12 +4768,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>62</v>
       </c>
       <c r="B64" t="n">
@@ -4805,12 +4793,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>63</v>
       </c>
       <c r="B65" t="n">
@@ -4830,12 +4818,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>64</v>
       </c>
       <c r="B66" t="n">
@@ -4855,12 +4843,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>65</v>
       </c>
       <c r="B67" t="n">
@@ -4880,12 +4868,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>66</v>
       </c>
       <c r="B68" t="n">
@@ -4905,12 +4893,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>67</v>
       </c>
       <c r="B69" t="n">
@@ -4930,12 +4918,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>68</v>
       </c>
       <c r="B70" t="n">
@@ -4955,12 +4943,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>69</v>
       </c>
       <c r="B71" t="n">
@@ -4980,12 +4968,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>70</v>
       </c>
       <c r="B72" t="n">
@@ -5005,12 +4993,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>71</v>
       </c>
       <c r="B73" t="n">
@@ -5030,12 +5018,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>72</v>
       </c>
       <c r="B74" t="n">
@@ -5055,12 +5043,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>73</v>
       </c>
       <c r="B75" t="n">
@@ -5080,12 +5068,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>74</v>
       </c>
       <c r="B76" t="n">
@@ -5105,12 +5093,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>75</v>
       </c>
       <c r="B77" t="n">
@@ -5130,12 +5118,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>76</v>
       </c>
       <c r="B78" t="n">
@@ -5155,12 +5143,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>77</v>
       </c>
       <c r="B79" t="n">
@@ -5180,12 +5168,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>78</v>
       </c>
       <c r="B80" t="n">
@@ -5205,12 +5193,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>79</v>
       </c>
       <c r="B81" t="n">
@@ -5230,12 +5218,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>80</v>
       </c>
       <c r="B82" t="n">
@@ -5255,12 +5243,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>81</v>
       </c>
       <c r="B83" t="n">
@@ -5280,12 +5268,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>82</v>
       </c>
       <c r="B84" t="n">
@@ -5305,12 +5293,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>83</v>
       </c>
       <c r="B85" t="n">
@@ -5330,12 +5318,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>84</v>
       </c>
       <c r="B86" t="n">
@@ -5355,12 +5343,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>85</v>
       </c>
       <c r="B87" t="n">
@@ -5380,12 +5368,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>86</v>
       </c>
       <c r="B88" t="n">
@@ -5405,12 +5393,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>87</v>
       </c>
       <c r="B89" t="n">
@@ -5430,12 +5418,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>88</v>
       </c>
       <c r="B90" t="n">
@@ -5455,12 +5443,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>89</v>
       </c>
       <c r="B91" t="n">
@@ -5480,12 +5468,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>90</v>
       </c>
       <c r="B92" t="n">
@@ -5505,12 +5493,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>91</v>
       </c>
       <c r="B93" t="n">
@@ -5530,12 +5518,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>92</v>
       </c>
       <c r="B94" t="n">
@@ -5555,12 +5543,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" t="n">
         <v>93</v>
       </c>
       <c r="B95" t="n">
@@ -5580,12 +5568,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" t="n">
         <v>94</v>
       </c>
       <c r="B96" t="n">
@@ -5605,12 +5593,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" t="n">
         <v>95</v>
       </c>
       <c r="B97" t="n">
@@ -5630,12 +5618,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" t="n">
         <v>96</v>
       </c>
       <c r="B98" t="n">
@@ -5655,12 +5643,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" t="n">
         <v>97</v>
       </c>
       <c r="B99" t="n">
@@ -5680,12 +5668,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" t="n">
         <v>98</v>
       </c>
       <c r="B100" t="n">
@@ -5705,12 +5693,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" t="n">
         <v>99</v>
       </c>
       <c r="B101" t="n">
@@ -5730,12 +5718,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" t="n">
         <v>100</v>
       </c>
       <c r="B102" t="n">
@@ -5755,7 +5743,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>C:\Users\NoahB\Documents\HebrewU Bioengineering\Cardiac_RODEO\Output\QC_Analysis\BucketAnalysis_QC_Range.xlsx</t>
+          <t>/Users/noahb/Documents/HebrewU Bioengineering/Cardiac_RODEO/Output/QC_Analysis/BucketAnalysis_QC_Range.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>